<commit_message>
Variante 3ch: monitor delle tensioni dei SiPM (ADC MCP3424 in I2C)
- partitori 1M/43k + 100n su VREG38 di ogni canale e sull'alta tensione
- ADC MCP3424 (U11, 0x68), resistenze serie 100R su SDA/SCL, connettore J6
- router: le linee MON stanno a >= 1,2 mm dai nodi analogici sensibili su
  entrambi gli strati (misurato: 1,6 mm); piste dei segnali invariate
- simulazione: con il monitor bias, impulsi e soglia restano identici
- software/monitor_tensioni.py per il Raspberry Pi
- footprint SOIC14 e HDR1x03, simboli MCP3424 e CONN3; stub dei SOIC dal lato lungo

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017fc9yPsNewCQrMK8R1c8Ls
</commit_message>
<xml_diff>
--- a/hardware/variante_3ch/jlcpcb/BOM_JLCPCB.xlsx
+++ b/hardware/variante_3ch/jlcpcb/BOM_JLCPCB.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -534,7 +534,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>C104,C121,C204,C221,C304,C321,CF4,CF7,CF8,CF9,CF11,CF101,CF102,CF105,CF106,CF110,CF201,CF202,CF205,CF206,CF210,CF301,CF302,CF305,CF306,CF310</t>
+          <t>C40,C104,C121,C150,C204,C221,C250,C304,C321,C350,CF4,CF7,CF8,CF9,CF11,CF12,CF101,CF102,CF105,CF106,CF110,CF201,CF202,CF205,CF206,CF210,CF301,CF302,CF305,CF306,CF310</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -777,12 +777,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0805W8F1201T5E</t>
+          <t>0805W8F1004T5E</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>R104,R204,R304</t>
+          <t>R40,R150,R250,R350</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -795,12 +795,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0805W8F1502T5E</t>
+          <t>0805W8F4302T5E</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>R105,R205,R305</t>
+          <t>R41,R151,R251,R351</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -813,12 +813,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0805W8F1003T5E</t>
+          <t>0805W8F1000T5E</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>R106,R120,R206,R220,R306,R320</t>
+          <t>R42,R43</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -831,12 +831,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0805W8F2702T5E</t>
+          <t>0805W8F1201T5E</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>R107,R207,R307</t>
+          <t>R104,R204,R304</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -849,12 +849,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0805W8F1001T5E</t>
+          <t>0805W8F1502T5E</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>R108,R112,R114,R115,R116,R208,R212,R214,R215,R216,R308,R312,R314,R315,R316</t>
+          <t>R105,R205,R305</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -867,12 +867,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0805W8F1801T5E</t>
+          <t>0805W8F1003T5E</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>R109,R209,R309</t>
+          <t>R106,R120,R206,R220,R306,R320</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -885,12 +885,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0805W8F5601T5E</t>
+          <t>0805W8F2702T5E</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>R111,R211,R311</t>
+          <t>R107,R207,R307</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -903,12 +903,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0805W8F5600T5E</t>
+          <t>0805W8F1001T5E</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>R113,R213,R313</t>
+          <t>R108,R112,R114,R115,R116,R208,R212,R214,R215,R216,R308,R312,R314,R315,R316</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -921,12 +921,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0805W8F4700T5E</t>
+          <t>0805W8F1801T5E</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>R117,R217,R317</t>
+          <t>R109,R209,R309</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -939,12 +939,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0805W8F100JT5E</t>
+          <t>0805W8F5601T5E</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>R118,R218,R318</t>
+          <t>R111,R211,R311</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -957,12 +957,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0805W8F1802T5E</t>
+          <t>0805W8F5600T5E</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>R119,R219,R319</t>
+          <t>R113,R213,R313</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -975,12 +975,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0805W8F820JT5E</t>
+          <t>0805W8F4700T5E</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>R121,R221,R321</t>
+          <t>R117,R217,R317</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -993,108 +993,184 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>MCP1825S-3302E/DB</t>
+          <t>0805W8F100JT5E</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>U6</t>
+          <t>R118,R218,R318</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>SOT-223</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>C148031</t>
-        </is>
-      </c>
+          <t>0805</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>SN74LVC1G11DBVR</t>
+          <t>0805W8F1802T5E</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>U10</t>
+          <t>R119,R219,R319</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>SOT-23-6</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>C22046</t>
-        </is>
-      </c>
+          <t>0805</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>TLC555CDR</t>
+          <t>0805W8F820JT5E</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>U102,U202,U302</t>
+          <t>R121,R221,R321</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>SOIC-8</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>C6986</t>
-        </is>
-      </c>
+          <t>0805</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>SN74LVC1G17DBVR</t>
+          <t>MCP1825S-3302E/DB</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>U109,U209,U309</t>
+          <t>U6</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>SOT-23-5</t>
+          <t>SOT-223</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>C7836</t>
+          <t>C148031</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>SN74LVC1G11DBVR</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>U10</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>SOT-23-6</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>C22046</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>MCP3424-E/SL</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>U11</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>SOIC-14</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>C640884</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>TLC555CDR</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>U102,U202,U302</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>SOIC-8</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>C6986</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>SN74LVC1G17DBVR</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>U109,U209,U309</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>SOT-23-5</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>C7836</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
           <t>3296W-1-103LF</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B38" t="inlineStr">
         <is>
           <t>V101,V102,V201,V202,V301,V302</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>3296W</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>C34846</t>
         </is>

</xml_diff>

<commit_message>
Scheda a 3 canali: protezione dell'alimentazione (USB-C, fusibile, TVS, MOSFET P, LED)
USB-C solo alimentazione J7 (GCT USB4125-GF-A, 5,1k su CC) o J3 da banco ->
fusibile ripristinabile F1 (MF-MSMF050-2) -> TVS D5 (SMAJ5.0A) -> MOSFET P Q4
(AO3401A, inversione di polarita') -> +5V; C60 10 uF e LED di accensione D6.
Generatore: piazzole con asola (guscio USB-C) in PCB KiCad, Gerber e foratura (G85);
nuovi simboli e impronte (dalla libreria KiCad 7.0.11); routing aggiunto senza toccare
le altre reti. Verifica KiCad: schema = PCB, DRC senza errori, 0 reti spezzate.
Simulazione ngspice della scheda intera: +5V 4,977 V, il resto invariato.
Schema A4: nuovo foglio 2 (ingresso e protezione); nota per il tecnico INFN aggiornata.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017fc9yPsNewCQrMK8R1c8Ls
</commit_message>
<xml_diff>
--- a/hardware/variante_3ch/jlcpcb/BOM_JLCPCB.xlsx
+++ b/hardware/variante_3ch/jlcpcb/BOM_JLCPCB.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:D49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -551,34 +551,34 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CL21B103KBANNNC</t>
+          <t>CL31B106KOHNNNE</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>C107,C111,C207,C211,C307,C311</t>
+          <t>C60</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0805</t>
+          <t>1206</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>C1710</t>
+          <t>C47971</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CL21C101JBANNNC</t>
+          <t>CL21B103KBANNNC</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>C109,C209,C309</t>
+          <t>C107,C111,C207,C211,C307,C311</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -588,19 +588,19 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>C1790</t>
+          <t>C1710</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CL21B225KAFNNNE</t>
+          <t>CL21C101JBANNNC</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CF4,CF7,CF9</t>
+          <t>C109,C209,C309</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -608,17 +608,21 @@
           <t>0805</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>C1790</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>NCD0805R1</t>
+          <t>CL21B225KAFNNNE</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>D103,D203,D303</t>
+          <t>CF4,CF7,CF9</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -626,199 +630,215 @@
           <t>0805</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>C84256</t>
-        </is>
-      </c>
+      <c r="D10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SRN5040-470M</t>
+          <t>SMAJ5.0A</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>SMD 5x5mm</t>
+          <t>SMA(DO-214AC)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>C1330294</t>
+          <t>C83329</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>BFR93AE6327HTSA1</t>
+          <t>KT-0805G</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Q101,Q201,Q301</t>
+          <t>D6</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>SOT-23</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>C513260</t>
+          <t>C2297</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MMBTH81</t>
+          <t>NCD0805R1</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Q102,Q202,Q302</t>
+          <t>D103,D203,D303</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>SOT-23</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>C190349</t>
+          <t>C84256</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0805W8F1002T5E</t>
+          <t>MF-MSMF050-2</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>R1,R31,R32,R33,R110,R152,R210,R252,R310,R352</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0805</t>
+          <t>1812</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>C17414</t>
+          <t>C17313</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0805W8F6802T5E</t>
+          <t>USB4125-GF-A</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>R2</t>
+          <t>J7</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>0805</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr"/>
+          <t>USB-C 6P SMD</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>C3151650</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0805W8F2553T5E</t>
+          <t>SRN5040-470M</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>0805</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr"/>
+          <t>SMD 5x5mm</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>C1330294</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0805W8F2203T5E</t>
+          <t>AO3401A</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>R22</t>
+          <t>Q4</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0805</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr"/>
+          <t>SOT-23</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>C15127</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0805W8F330JT5E</t>
+          <t>BFR93AE6327HTSA1</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>R30,R123,R223,R323</t>
+          <t>Q101,Q201,Q301</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0805</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr"/>
+          <t>SOT-23</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>C513260</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0805W8F1004T5E</t>
+          <t>MMBTH81</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>R40,R150,R250,R350</t>
+          <t>Q102,Q202,Q302</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0805</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr"/>
+          <t>SOT-23</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>C190349</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0805W8F4302T5E</t>
+          <t>0805W8F1002T5E</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>R41,R151,R251,R351</t>
+          <t>R1,R31,R32,R33,R62,R110,R152,R210,R252,R310,R352</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -826,17 +846,21 @@
           <t>0805</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>C17414</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0805W8F1000T5E</t>
+          <t>0805W8F6802T5E</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>R42,R43</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -849,12 +873,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0805W8F2202T5E</t>
+          <t>0805W8F2553T5E</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>R44</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -867,12 +891,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0805W8F1201T5E</t>
+          <t>0805W8F2203T5E</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>R104,R204,R304</t>
+          <t>R22</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -885,12 +909,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0805W8F1502T5E</t>
+          <t>0805W8F330JT5E</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>R105,R205,R305</t>
+          <t>R30,R123,R223,R323</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -903,12 +927,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0805W8F1003T5E</t>
+          <t>0805W8F1004T5E</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>R106,R120,R206,R220,R306,R320</t>
+          <t>R40,R150,R250,R350</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -921,12 +945,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0805W8F2702T5E</t>
+          <t>0805W8F4302T5E</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>R107,R207,R307</t>
+          <t>R41,R151,R251,R351</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -939,12 +963,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0805W8F1001T5E</t>
+          <t>0805W8F1000T5E</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>R108,R112,R114,R115,R116,R208,R212,R214,R215,R216,R308,R312,R314,R315,R316</t>
+          <t>R42,R43</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -957,12 +981,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0805W8F1801T5E</t>
+          <t>0805W8F2202T5E</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>R109,R209,R309</t>
+          <t>R44</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -975,12 +999,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0805W8F5601T5E</t>
+          <t>0805W8F5101T5E</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>R111,R211,R311</t>
+          <t>R60,R61</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -993,12 +1017,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0805W8F5600T5E</t>
+          <t>0805W8F1501T5E</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>R113,R213,R313</t>
+          <t>R63</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1011,12 +1035,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0805W8F4700T5E</t>
+          <t>0805W8F1201T5E</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>R117,R217,R317</t>
+          <t>R104,R204,R304</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1029,12 +1053,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>0805W8F100JT5E</t>
+          <t>0805W8F1502T5E</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>R118,R218,R318</t>
+          <t>R105,R205,R305</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1047,12 +1071,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0805W8F1802T5E</t>
+          <t>0805W8F1003T5E</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>R119,R219,R319</t>
+          <t>R106,R120,R206,R220,R306,R320</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1065,12 +1089,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>0805W8F820JT5E</t>
+          <t>0805W8F2702T5E</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>R121,R221,R321</t>
+          <t>R107,R207,R307</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1083,12 +1107,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>NCP21XV103J03RA</t>
+          <t>0805W8F1001T5E</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>RT1</t>
+          <t>R108,R112,R114,R115,R116,R208,R212,R214,R215,R216,R308,R312,R314,R315,R316</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1101,130 +1125,274 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>MCP1825S-3302E/DB</t>
+          <t>0805W8F1801T5E</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>U6</t>
+          <t>R109,R209,R309</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>SOT-223</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>C148031</t>
-        </is>
-      </c>
+          <t>0805</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SN74LVC1G11DBVR</t>
+          <t>0805W8F5601T5E</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>U10</t>
+          <t>R111,R211,R311</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>SOT-23-6</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>C22046</t>
-        </is>
-      </c>
+          <t>0805</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>MCP3424-E/SL</t>
+          <t>0805W8F5600T5E</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>U11,U12</t>
+          <t>R113,R213,R313</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>SOIC-14</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>C640884</t>
-        </is>
-      </c>
+          <t>0805</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>TLC555CDR</t>
+          <t>0805W8F4700T5E</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>U102,U202,U302</t>
+          <t>R117,R217,R317</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>SOIC-8</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>C6986</t>
-        </is>
-      </c>
+          <t>0805</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>SN74LVC1G17DBVR</t>
+          <t>0805W8F100JT5E</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>U109,U209,U309</t>
+          <t>R118,R218,R318</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>SOT-23-5</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>C7836</t>
-        </is>
-      </c>
+          <t>0805</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>0805W8F1802T5E</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>R119,R219,R319</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>0805</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>0805W8F820JT5E</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>R121,R221,R321</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>0805</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>NCP21XV103J03RA</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>RT1</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>0805</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>MCP1825S-3302E/DB</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>U6</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>SOT-223</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>C148031</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>SN74LVC1G11DBVR</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>U10</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>SOT-23-6</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>C22046</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>MCP3424-E/SL</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>U11,U12</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>SOIC-14</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>C640884</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>TLC555CDR</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>U102,U202,U302</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>SOIC-8</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>C6986</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>SN74LVC1G17DBVR</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>U109,U209,U309</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>SOT-23-5</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>C7836</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
           <t>3296W-1-103LF</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B49" t="inlineStr">
         <is>
           <t>V101,V102,V201,V202,V301,V302</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>3296W</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D49" t="inlineStr">
         <is>
           <t>C34846</t>
         </is>

</xml_diff>